<commit_message>
Udpated power sector calibration to use suggested NEXT Group retirements for coal, update capacity retirements based NEXT Group data, update RPS based on policy language, and remove CES.
</commit_message>
<xml_diff>
--- a/InputData/elec/BPMCCS/BAU Pol Mandated Cap Const Sched.xlsx
+++ b/InputData/elec/BPMCCS/BAU Pol Mandated Cap Const Sched.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\South Korea\Models\eps-southkorea\InputData\elec\BPMCCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF249023-3B75-4723-847B-C8191E189920}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CFB81C3-6986-46A3-B05D-B75EF1AC9D8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6825" yWindow="4485" windowWidth="17280" windowHeight="10005" tabRatio="846" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="465" yWindow="795" windowWidth="25770" windowHeight="20955" tabRatio="846" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="6" r:id="rId1"/>
@@ -783,10 +783,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>*2021년도 값 제외하기</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>&lt; 연도별 풍력·태양광 보급 (단위: MW) &gt;</t>
   </si>
   <si>
@@ -812,6 +808,9 @@
   </si>
   <si>
     <t>2026-09-04: hydro 2025 mandated build (1,815 MW) removed - the source cell was the cumulative conventional hydro fleet total, not an addition. EPS hydro capacity had jumped 2.1 -&gt; 3.9 GW in 2025 (actual fleet ~1.8 GW).</t>
+  </si>
+  <si>
+    <t>2026-09-14 partner round 2 file adopted (260911): hard coal 2021 mandated build 3,098 MW (Goseong Hai 1-2 2,080 MW, Shin-Seocheon 1 1,018 MW) added in the 설비현황 tab. Consistent with the start-year convention: BHRaSYC hard coal is the end-2020 fleet (rebuilt from the EPSIS unit list the same day), so 2021 = end-2020 fleet + this build - the 2,620 MW retired in BCRbQ 2021 = 36.97 GW vs KPX 36.94 GW.</t>
   </si>
 </sst>
 </file>
@@ -993,7 +992,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1087,6 +1086,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9D9D9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF7979"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1406,7 +1411,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="108">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1613,6 +1618,7 @@
     </xf>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2035,6 +2041,11 @@
         <v>31</v>
       </c>
     </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>220</v>
+      </c>
+    </row>
     <row r="3" spans="1:2">
       <c r="A3" s="4" t="s">
         <v>32</v>
@@ -2128,7 +2139,7 @@
     </row>
     <row r="26" spans="1:1">
       <c r="A26" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="27" spans="1:1">
@@ -2136,7 +2147,7 @@
     </row>
     <row r="28" spans="1:1">
       <c r="A28" s="1" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="29" spans="1:1">
@@ -3096,12 +3107,12 @@
     </row>
     <row r="103" spans="1:17">
       <c r="A103" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="104" spans="1:17">
       <c r="A104" s="92" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B104" s="93">
         <v>2023</v>
@@ -3326,12 +3337,12 @@
     </row>
     <row r="109" spans="1:17">
       <c r="A109" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="110" spans="1:17">
       <c r="A110" s="92" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B110" s="92" t="s">
         <v>97</v>
@@ -3340,7 +3351,7 @@
         <v>111</v>
       </c>
       <c r="D110" s="92" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E110" s="92" t="s">
         <v>112</v>
@@ -3349,7 +3360,7 @@
         <v>95</v>
       </c>
       <c r="G110" s="92" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="H110" s="92" t="s">
         <v>101</v>
@@ -3357,7 +3368,7 @@
     </row>
     <row r="111" spans="1:17">
       <c r="A111" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B111" s="95">
         <v>0</v>
@@ -3723,8 +3734,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="D25" s="49">
-        <v>0</v>
+      <c r="D25" s="96">
+        <f t="shared" si="0"/>
+        <v>3098</v>
       </c>
       <c r="E25" s="7">
         <f t="shared" si="0"/>
@@ -3742,9 +3754,6 @@
         <f t="shared" si="0"/>
         <v>1050</v>
       </c>
-      <c r="I25" t="s">
-        <v>211</v>
-      </c>
     </row>
     <row r="26" spans="1:10">
       <c r="A26" s="7" t="s">
@@ -3843,7 +3852,7 @@
         <v>7</v>
       </c>
       <c r="B29" s="7">
-        <f t="shared" ref="B29:H29" si="3">C6</f>
+        <f t="shared" ref="B29:G29" si="3">C6</f>
         <v>0</v>
       </c>
       <c r="C29" s="7">
@@ -3870,7 +3879,7 @@
         <v>0</v>
       </c>
       <c r="J29" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="30" spans="1:10">
@@ -4460,51 +4469,51 @@
       </c>
     </row>
     <row r="5" spans="1:13">
-      <c r="A5" s="98" t="s">
-        <v>0</v>
-      </c>
-      <c r="B5" s="101" t="s">
+      <c r="A5" s="99" t="s">
+        <v>0</v>
+      </c>
+      <c r="B5" s="102" t="s">
         <v>108</v>
       </c>
-      <c r="C5" s="101"/>
-      <c r="D5" s="101"/>
-      <c r="E5" s="101"/>
-      <c r="F5" s="101"/>
-      <c r="G5" s="101"/>
-      <c r="H5" s="101"/>
-      <c r="I5" s="101"/>
-      <c r="J5" s="101"/>
-      <c r="K5" s="101"/>
-      <c r="L5" s="101" t="s">
+      <c r="C5" s="102"/>
+      <c r="D5" s="102"/>
+      <c r="E5" s="102"/>
+      <c r="F5" s="102"/>
+      <c r="G5" s="102"/>
+      <c r="H5" s="102"/>
+      <c r="I5" s="102"/>
+      <c r="J5" s="102"/>
+      <c r="K5" s="102"/>
+      <c r="L5" s="102" t="s">
         <v>109</v>
       </c>
-      <c r="M5" s="104" t="s">
+      <c r="M5" s="105" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="6" spans="1:13">
-      <c r="A6" s="99"/>
-      <c r="B6" s="102" t="s">
+      <c r="A6" s="100"/>
+      <c r="B6" s="103" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="102"/>
-      <c r="D6" s="102"/>
-      <c r="E6" s="102"/>
-      <c r="F6" s="102"/>
-      <c r="G6" s="102"/>
-      <c r="H6" s="102" t="s">
+      <c r="C6" s="103"/>
+      <c r="D6" s="103"/>
+      <c r="E6" s="103"/>
+      <c r="F6" s="103"/>
+      <c r="G6" s="103"/>
+      <c r="H6" s="103" t="s">
         <v>5</v>
       </c>
-      <c r="I6" s="102"/>
-      <c r="J6" s="102"/>
-      <c r="K6" s="102" t="s">
+      <c r="I6" s="103"/>
+      <c r="J6" s="103"/>
+      <c r="K6" s="103" t="s">
         <v>110</v>
       </c>
-      <c r="L6" s="102"/>
-      <c r="M6" s="105"/>
+      <c r="L6" s="103"/>
+      <c r="M6" s="106"/>
     </row>
     <row r="7" spans="1:13" ht="15.75" thickBot="1">
-      <c r="A7" s="100"/>
+      <c r="A7" s="101"/>
       <c r="B7" s="24" t="s">
         <v>97</v>
       </c>
@@ -4532,12 +4541,12 @@
       <c r="J7" s="24" t="s">
         <v>113</v>
       </c>
-      <c r="K7" s="103"/>
-      <c r="L7" s="103"/>
-      <c r="M7" s="106"/>
+      <c r="K7" s="104"/>
+      <c r="L7" s="104"/>
+      <c r="M7" s="107"/>
     </row>
     <row r="8" spans="1:13">
-      <c r="A8" s="107">
+      <c r="A8" s="108">
         <v>2024</v>
       </c>
       <c r="B8" s="22">
@@ -4578,7 +4587,7 @@
       </c>
     </row>
     <row r="9" spans="1:13">
-      <c r="A9" s="96"/>
+      <c r="A9" s="97"/>
       <c r="B9" s="17">
         <v>4025</v>
       </c>
@@ -4613,7 +4622,7 @@
       <c r="M9" s="20"/>
     </row>
     <row r="10" spans="1:13">
-      <c r="A10" s="96">
+      <c r="A10" s="97">
         <v>2025</v>
       </c>
       <c r="B10" s="16">
@@ -4654,7 +4663,7 @@
       </c>
     </row>
     <row r="11" spans="1:13">
-      <c r="A11" s="96"/>
+      <c r="A11" s="97"/>
       <c r="B11" s="17">
         <v>4571</v>
       </c>
@@ -4689,7 +4698,7 @@
       <c r="M11" s="20"/>
     </row>
     <row r="12" spans="1:13">
-      <c r="A12" s="96">
+      <c r="A12" s="97">
         <v>2026</v>
       </c>
       <c r="B12" s="16">
@@ -4730,7 +4739,7 @@
       </c>
     </row>
     <row r="13" spans="1:13">
-      <c r="A13" s="96"/>
+      <c r="A13" s="97"/>
       <c r="B13" s="17">
         <v>5161</v>
       </c>
@@ -4765,7 +4774,7 @@
       <c r="M13" s="20"/>
     </row>
     <row r="14" spans="1:13">
-      <c r="A14" s="96">
+      <c r="A14" s="97">
         <v>2027</v>
       </c>
       <c r="B14" s="16">
@@ -4806,7 +4815,7 @@
       </c>
     </row>
     <row r="15" spans="1:13">
-      <c r="A15" s="96"/>
+      <c r="A15" s="97"/>
       <c r="B15" s="17">
         <v>5780</v>
       </c>
@@ -4841,7 +4850,7 @@
       <c r="M15" s="20"/>
     </row>
     <row r="16" spans="1:13">
-      <c r="A16" s="96">
+      <c r="A16" s="97">
         <v>2028</v>
       </c>
       <c r="B16" s="16">
@@ -4882,7 +4891,7 @@
       </c>
     </row>
     <row r="17" spans="1:13">
-      <c r="A17" s="96"/>
+      <c r="A17" s="97"/>
       <c r="B17" s="17">
         <v>6409</v>
       </c>
@@ -4917,7 +4926,7 @@
       <c r="M17" s="20"/>
     </row>
     <row r="18" spans="1:13">
-      <c r="A18" s="96">
+      <c r="A18" s="97">
         <v>2029</v>
       </c>
       <c r="B18" s="16">
@@ -4958,7 +4967,7 @@
       </c>
     </row>
     <row r="19" spans="1:13">
-      <c r="A19" s="96"/>
+      <c r="A19" s="97"/>
       <c r="B19" s="17">
         <v>7046</v>
       </c>
@@ -4993,7 +5002,7 @@
       <c r="M19" s="20"/>
     </row>
     <row r="20" spans="1:13">
-      <c r="A20" s="96">
+      <c r="A20" s="97">
         <v>2030</v>
       </c>
       <c r="B20" s="16">
@@ -5034,7 +5043,7 @@
       </c>
     </row>
     <row r="21" spans="1:13">
-      <c r="A21" s="96"/>
+      <c r="A21" s="97"/>
       <c r="B21" s="17">
         <v>7962</v>
       </c>
@@ -5069,7 +5078,7 @@
       <c r="M21" s="20"/>
     </row>
     <row r="22" spans="1:13">
-      <c r="A22" s="96">
+      <c r="A22" s="97">
         <v>2031</v>
       </c>
       <c r="B22" s="16">
@@ -5110,7 +5119,7 @@
       </c>
     </row>
     <row r="23" spans="1:13">
-      <c r="A23" s="96"/>
+      <c r="A23" s="97"/>
       <c r="B23" s="17">
         <v>8396</v>
       </c>
@@ -5145,7 +5154,7 @@
       <c r="M23" s="20"/>
     </row>
     <row r="24" spans="1:13">
-      <c r="A24" s="96">
+      <c r="A24" s="97">
         <v>2032</v>
       </c>
       <c r="B24" s="16">
@@ -5186,7 +5195,7 @@
       </c>
     </row>
     <row r="25" spans="1:13">
-      <c r="A25" s="96"/>
+      <c r="A25" s="97"/>
       <c r="B25" s="17">
         <v>8829</v>
       </c>
@@ -5221,7 +5230,7 @@
       <c r="M25" s="20"/>
     </row>
     <row r="26" spans="1:13">
-      <c r="A26" s="96">
+      <c r="A26" s="97">
         <v>2033</v>
       </c>
       <c r="B26" s="16">
@@ -5262,7 +5271,7 @@
       </c>
     </row>
     <row r="27" spans="1:13">
-      <c r="A27" s="96"/>
+      <c r="A27" s="97"/>
       <c r="B27" s="17">
         <v>9261</v>
       </c>
@@ -5297,7 +5306,7 @@
       <c r="M27" s="20"/>
     </row>
     <row r="28" spans="1:13">
-      <c r="A28" s="96">
+      <c r="A28" s="97">
         <v>2034</v>
       </c>
       <c r="B28" s="16">
@@ -5338,7 +5347,7 @@
       </c>
     </row>
     <row r="29" spans="1:13">
-      <c r="A29" s="96"/>
+      <c r="A29" s="97"/>
       <c r="B29" s="17">
         <v>9693</v>
       </c>
@@ -5373,7 +5382,7 @@
       <c r="M29" s="20"/>
     </row>
     <row r="30" spans="1:13">
-      <c r="A30" s="96">
+      <c r="A30" s="97">
         <v>2035</v>
       </c>
       <c r="B30" s="16">
@@ -5414,7 +5423,7 @@
       </c>
     </row>
     <row r="31" spans="1:13">
-      <c r="A31" s="96"/>
+      <c r="A31" s="97"/>
       <c r="B31" s="17">
         <v>10126</v>
       </c>
@@ -5449,7 +5458,7 @@
       <c r="M31" s="20"/>
     </row>
     <row r="32" spans="1:13">
-      <c r="A32" s="96">
+      <c r="A32" s="97">
         <v>2036</v>
       </c>
       <c r="B32" s="16">
@@ -5490,7 +5499,7 @@
       </c>
     </row>
     <row r="33" spans="1:17">
-      <c r="A33" s="96"/>
+      <c r="A33" s="97"/>
       <c r="B33" s="17">
         <v>10431</v>
       </c>
@@ -5525,7 +5534,7 @@
       <c r="M33" s="20"/>
     </row>
     <row r="34" spans="1:17">
-      <c r="A34" s="96">
+      <c r="A34" s="97">
         <v>2037</v>
       </c>
       <c r="B34" s="16">
@@ -5566,7 +5575,7 @@
       </c>
     </row>
     <row r="35" spans="1:17">
-      <c r="A35" s="96"/>
+      <c r="A35" s="97"/>
       <c r="B35" s="17">
         <v>10735</v>
       </c>
@@ -5601,7 +5610,7 @@
       <c r="M35" s="20"/>
     </row>
     <row r="36" spans="1:17">
-      <c r="A36" s="96">
+      <c r="A36" s="97">
         <v>2038</v>
       </c>
       <c r="B36" s="16">
@@ -5642,7 +5651,7 @@
       </c>
     </row>
     <row r="37" spans="1:17" ht="15.75" thickBot="1">
-      <c r="A37" s="97"/>
+      <c r="A37" s="98"/>
       <c r="B37" s="18">
         <v>11040</v>
       </c>
@@ -9916,7 +9925,7 @@
       </c>
       <c r="D2" s="76">
         <f>'설비현황_19~25'!D25</f>
-        <v>0</v>
+        <v>3098</v>
       </c>
       <c r="E2" s="76">
         <f>'설비현황_19~25'!E25</f>
@@ -13095,20 +13104,12 @@
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="688c5d3b-a76a-458b-b159-91c2a1154680">
@@ -13118,7 +13119,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="문서" ma:contentTypeID="0x01010027350D42B0D95040ACC873ED5DCB146E" ma:contentTypeVersion="10" ma:contentTypeDescription="새 문서를 만듭니다." ma:contentTypeScope="" ma:versionID="c2e4f52adf7af47ba555973ff8cbcabe">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="688c5d3b-a76a-458b-b159-91c2a1154680" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="502e33886199ad3dabc1cc93359c84e5" ns2:_="">
     <xsd:import namespace="688c5d3b-a76a-458b-b159-91c2a1154680"/>
@@ -13294,15 +13295,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5AC0E8B6-FC6C-47AD-8E91-EBF41CCB1712}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13444BB4-D2AE-4704-9F59-09418FDD2FE0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -13312,7 +13314,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C8EFB68-B099-4082-B802-B144AFACC6EB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -13330,6 +13332,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5AC0E8B6-FC6C-47AD-8E91-EBF41CCB1712}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{c7ef1c8b-ba63-4702-8e74-5094387a97de}" enabled="0" method="" siteId="{c7ef1c8b-ba63-4702-8e74-5094387a97de}" removed="1"/>

</xml_diff>